<commit_message>
Sincronizaci├│n autom├ítica 31/01/2026 12:49:37.85
</commit_message>
<xml_diff>
--- a/Fichas/Q037.xlsx
+++ b/Fichas/Q037.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27818"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\CONTROL DISEÑO\VIVA ROUSS\QPTIMA 2025\DESAROLLOS 25\Q037 CROP TOP TEEN CON CINTAS EN LA SIZA Y CUELLO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\DESKTOP-ID9UEKK\Users\Admin\Desktop\CONTROL DISEÑO\VIVA ROUSS\QPTIMA 2025\DESAROLLOS 25\Q037 CROP TOP TEEN CON CINTAS EN LA SIZA Y CUELLO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447EB19D-BA25-44C5-A048-6F9635203817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DCA8930-9CD0-4113-AA53-A5F1A3B7E081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FICHA TECNICA" sheetId="1" r:id="rId1"/>
     <sheet name="CONFECCION" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="72">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -79,44 +79,12 @@
     <t>ENHEBRADO</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>SIS.</t>
   </si>
   <si>
     <t>TIPO DE MAQUINA</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>G</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>HILO</t>
-    </r>
-  </si>
-  <si>
     <t>NYLON</t>
   </si>
   <si>
@@ -144,18 +112,6 @@
     <t>CROP TOP TEEN SIZADO CUELLO REDONDO</t>
   </si>
   <si>
-    <t>LICRA DESNUDA</t>
-  </si>
-  <si>
-    <t>#3</t>
-  </si>
-  <si>
-    <t>2 Y 6</t>
-  </si>
-  <si>
-    <t>Q037B31M</t>
-  </si>
-  <si>
     <t>Q037TUBO</t>
   </si>
   <si>
@@ -225,9 +181,6 @@
     <t>T-CH</t>
   </si>
   <si>
-    <t>CH</t>
-  </si>
-  <si>
     <t>MAQUINA</t>
   </si>
   <si>
@@ -265,6 +218,39 @@
   </si>
   <si>
     <t>INCLUYE  CINTA DE LA COLLARETA</t>
+  </si>
+  <si>
+    <t>GRANDE</t>
+  </si>
+  <si>
+    <t>CHICA</t>
+  </si>
+  <si>
+    <t>MEDIANA</t>
+  </si>
+  <si>
+    <t>Q037B31G</t>
+  </si>
+  <si>
+    <t>Q037B08M</t>
+  </si>
+  <si>
+    <t>Q037B13C</t>
+  </si>
+  <si>
+    <t>GH</t>
+  </si>
+  <si>
+    <t>TOP2</t>
+  </si>
+  <si>
+    <t>EVO</t>
+  </si>
+  <si>
+    <t>#7</t>
+  </si>
+  <si>
+    <t>MAQ#31</t>
   </si>
 </sst>
 </file>
@@ -307,20 +293,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="24"/>
-      <color rgb="FFFFFF00"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FFFFFF00"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -333,19 +305,6 @@
       <family val="3"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="20"/>
-      <color rgb="FFFFFF00"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
       <b/>
       <sz val="18"/>
       <name val="Consolas"/>
@@ -353,29 +312,7 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <b/>
       <sz val="14"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="22"/>
       <name val="Consolas"/>
       <family val="3"/>
     </font>
@@ -386,42 +323,10 @@
       <family val="3"/>
     </font>
     <font>
-      <sz val="18"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="16"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="22"/>
-      <color rgb="FF000000"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <sz val="20"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="26"/>
-      <color rgb="FF000000"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
     <font>
       <sz val="11"/>
@@ -499,8 +404,103 @@
       <name val="Arial Black"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="28"/>
+      <color theme="0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="26"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14.5"/>
+      <color theme="0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color theme="0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -553,6 +553,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -760,9 +766,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="23" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -786,357 +792,366 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="22" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="31" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="31" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="26" fillId="7" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="26" fillId="7" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="26" fillId="7" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="26" fillId="7" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="7" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="7" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="36" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="36" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="28" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="28" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="28" fillId="10" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="28" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="36" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="7" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="7" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="7" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="7" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="19" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="19" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="20" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="20" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="20" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="35" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="21" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1239,14 +1254,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>28576</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>219075</xdr:rowOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>686420</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>14625</xdr:rowOff>
+      <xdr:colOff>657226</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>24149</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1274,8 +1289,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="66676" y="781050"/>
-          <a:ext cx="1457944" cy="1872000"/>
+          <a:off x="66676" y="1190625"/>
+          <a:ext cx="1428750" cy="2376824"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1637,7 +1652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O780"/>
+  <dimension ref="A1:R778"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="0.5703125" customWidth="1"/>
@@ -1645,19 +1660,21 @@
     <col min="3" max="3" width="5.28515625" customWidth="1"/>
     <col min="4" max="4" width="10.7109375" customWidth="1"/>
     <col min="5" max="5" width="6.5703125" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" customWidth="1"/>
-    <col min="9" max="9" width="5.7109375" customWidth="1"/>
-    <col min="10" max="10" width="9.7109375" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" customWidth="1"/>
-    <col min="12" max="12" width="5.7109375" customWidth="1"/>
-    <col min="13" max="13" width="9.7109375" customWidth="1"/>
-    <col min="14" max="14" width="10.7109375" customWidth="1"/>
-    <col min="15" max="15" width="5.7109375" customWidth="1"/>
+    <col min="6" max="7" width="6.7109375" customWidth="1"/>
+    <col min="8" max="8" width="8.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.28515625" customWidth="1"/>
+    <col min="10" max="10" width="6.7109375" customWidth="1"/>
+    <col min="11" max="11" width="8.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.28515625" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.7109375" customWidth="1"/>
+    <col min="15" max="15" width="4.28515625" customWidth="1"/>
+    <col min="16" max="16" width="6.7109375" customWidth="1"/>
+    <col min="17" max="17" width="8.7109375" customWidth="1"/>
+    <col min="18" max="18" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="1.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1675,581 +1692,687 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
-    </row>
-    <row r="2" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="49" t="s">
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+    </row>
+    <row r="2" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="50"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="78" t="s">
+      <c r="C2" s="54"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="75" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
-      <c r="L2" s="78"/>
-      <c r="M2" s="78"/>
-      <c r="N2" s="78"/>
-      <c r="O2" s="79"/>
-    </row>
-    <row r="3" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="52"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
-      <c r="J3" s="80"/>
-      <c r="K3" s="80"/>
-      <c r="L3" s="80"/>
-      <c r="M3" s="80"/>
-      <c r="N3" s="80"/>
-      <c r="O3" s="81"/>
-    </row>
-    <row r="4" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
+      <c r="L2" s="75"/>
+      <c r="M2" s="75"/>
+      <c r="N2" s="75"/>
+      <c r="O2" s="75"/>
+      <c r="P2" s="75"/>
+      <c r="Q2" s="75"/>
+      <c r="R2" s="76"/>
+    </row>
+    <row r="3" spans="1:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="56"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="77"/>
+      <c r="J3" s="77"/>
+      <c r="K3" s="77"/>
+      <c r="L3" s="77"/>
+      <c r="M3" s="77"/>
+      <c r="N3" s="77"/>
+      <c r="O3" s="77"/>
+      <c r="P3" s="77"/>
+      <c r="Q3" s="77"/>
+      <c r="R3" s="78"/>
+    </row>
+    <row r="4" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
-      <c r="E4" s="106" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" s="107"/>
-      <c r="G4" s="107"/>
-      <c r="H4" s="107"/>
-      <c r="I4" s="107"/>
-      <c r="J4" s="107"/>
-      <c r="K4" s="107"/>
-      <c r="L4" s="107"/>
-      <c r="M4" s="107"/>
-      <c r="N4" s="107"/>
-      <c r="O4" s="108"/>
-    </row>
-    <row r="5" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E4" s="119" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="120"/>
+      <c r="G4" s="120"/>
+      <c r="H4" s="120"/>
+      <c r="I4" s="120"/>
+      <c r="J4" s="120"/>
+      <c r="K4" s="120"/>
+      <c r="L4" s="120"/>
+      <c r="M4" s="120"/>
+      <c r="N4" s="120"/>
+      <c r="O4" s="120"/>
+      <c r="P4" s="120"/>
+      <c r="Q4" s="120"/>
+      <c r="R4" s="121"/>
+    </row>
+    <row r="5" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
       <c r="C5" s="5"/>
       <c r="D5" s="7"/>
-      <c r="E5" s="109"/>
-      <c r="F5" s="110"/>
-      <c r="G5" s="110"/>
-      <c r="H5" s="110"/>
-      <c r="I5" s="110"/>
-      <c r="J5" s="110"/>
-      <c r="K5" s="110"/>
-      <c r="L5" s="110"/>
-      <c r="M5" s="110"/>
-      <c r="N5" s="110"/>
-      <c r="O5" s="111"/>
-    </row>
-    <row r="6" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E5" s="122"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="123"/>
+      <c r="H5" s="123"/>
+      <c r="I5" s="123"/>
+      <c r="J5" s="123"/>
+      <c r="K5" s="123"/>
+      <c r="L5" s="123"/>
+      <c r="M5" s="123"/>
+      <c r="N5" s="123"/>
+      <c r="O5" s="123"/>
+      <c r="P5" s="123"/>
+      <c r="Q5" s="123"/>
+      <c r="R5" s="124"/>
+    </row>
+    <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2"/>
       <c r="C6" s="5"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="109"/>
-      <c r="F6" s="110"/>
-      <c r="G6" s="110"/>
-      <c r="H6" s="110"/>
-      <c r="I6" s="110"/>
-      <c r="J6" s="110"/>
-      <c r="K6" s="110"/>
-      <c r="L6" s="110"/>
-      <c r="M6" s="110"/>
-      <c r="N6" s="110"/>
-      <c r="O6" s="111"/>
-    </row>
-    <row r="7" spans="1:15" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E6" s="122"/>
+      <c r="F6" s="123"/>
+      <c r="G6" s="123"/>
+      <c r="H6" s="123"/>
+      <c r="I6" s="123"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
+      <c r="L6" s="123"/>
+      <c r="M6" s="123"/>
+      <c r="N6" s="123"/>
+      <c r="O6" s="123"/>
+      <c r="P6" s="123"/>
+      <c r="Q6" s="123"/>
+      <c r="R6" s="124"/>
+    </row>
+    <row r="7" spans="1:18" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2"/>
       <c r="C7" s="5"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
-      <c r="H7" s="113"/>
-      <c r="I7" s="113"/>
-      <c r="J7" s="113"/>
-      <c r="K7" s="113"/>
-      <c r="L7" s="113"/>
-      <c r="M7" s="113"/>
-      <c r="N7" s="113"/>
-      <c r="O7" s="114"/>
-    </row>
-    <row r="8" spans="1:15" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E7" s="125"/>
+      <c r="F7" s="126"/>
+      <c r="G7" s="126"/>
+      <c r="H7" s="126"/>
+      <c r="I7" s="126"/>
+      <c r="J7" s="126"/>
+      <c r="K7" s="126"/>
+      <c r="L7" s="126"/>
+      <c r="M7" s="126"/>
+      <c r="N7" s="126"/>
+      <c r="O7" s="126"/>
+      <c r="P7" s="126"/>
+      <c r="Q7" s="126"/>
+      <c r="R7" s="127"/>
+    </row>
+    <row r="8" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2"/>
       <c r="C8" s="5"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="37" t="s">
+      <c r="E8" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="38"/>
-      <c r="G8" s="92" t="s">
-        <v>54</v>
-      </c>
-      <c r="H8" s="93"/>
-      <c r="I8" s="94"/>
-      <c r="J8" s="92"/>
-      <c r="K8" s="93"/>
-      <c r="L8" s="94"/>
-      <c r="M8" s="92" t="s">
-        <v>14</v>
-      </c>
-      <c r="N8" s="93"/>
-      <c r="O8" s="94"/>
-    </row>
-    <row r="9" spans="1:15" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F8" s="42"/>
+      <c r="G8" s="107" t="s">
+        <v>62</v>
+      </c>
+      <c r="H8" s="108"/>
+      <c r="I8" s="109"/>
+      <c r="J8" s="107" t="s">
+        <v>63</v>
+      </c>
+      <c r="K8" s="108"/>
+      <c r="L8" s="109"/>
+      <c r="M8" s="107" t="s">
+        <v>61</v>
+      </c>
+      <c r="N8" s="108"/>
+      <c r="O8" s="109"/>
+      <c r="P8" s="89" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q8" s="90"/>
+      <c r="R8" s="91"/>
+    </row>
+    <row r="9" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2"/>
       <c r="C9" s="5"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="95"/>
-      <c r="H9" s="96"/>
-      <c r="I9" s="97"/>
-      <c r="J9" s="95"/>
-      <c r="K9" s="96"/>
-      <c r="L9" s="97"/>
-      <c r="M9" s="95"/>
-      <c r="N9" s="96"/>
-      <c r="O9" s="97"/>
-    </row>
-    <row r="10" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E9" s="41"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="110"/>
+      <c r="H9" s="111"/>
+      <c r="I9" s="112"/>
+      <c r="J9" s="110"/>
+      <c r="K9" s="111"/>
+      <c r="L9" s="112"/>
+      <c r="M9" s="110"/>
+      <c r="N9" s="111"/>
+      <c r="O9" s="112"/>
+      <c r="P9" s="92"/>
+      <c r="Q9" s="93"/>
+      <c r="R9" s="94"/>
+    </row>
+    <row r="10" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2"/>
       <c r="C10" s="5"/>
       <c r="D10" s="7"/>
-      <c r="E10" s="37" t="s">
+      <c r="E10" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="F10" s="38"/>
-      <c r="G10" s="98" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" s="99"/>
-      <c r="I10" s="100"/>
-      <c r="J10" s="98" t="s">
-        <v>32</v>
-      </c>
-      <c r="K10" s="99"/>
-      <c r="L10" s="100"/>
-      <c r="M10" s="98" t="s">
-        <v>14</v>
-      </c>
-      <c r="N10" s="99"/>
-      <c r="O10" s="100"/>
-    </row>
-    <row r="11" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F10" s="42"/>
+      <c r="G10" s="97" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" s="98"/>
+      <c r="I10" s="98"/>
+      <c r="J10" s="98"/>
+      <c r="K10" s="98"/>
+      <c r="L10" s="98"/>
+      <c r="M10" s="98"/>
+      <c r="N10" s="98"/>
+      <c r="O10" s="99"/>
+      <c r="P10" s="89" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q10" s="90"/>
+      <c r="R10" s="91"/>
+    </row>
+    <row r="11" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2"/>
       <c r="C11" s="5"/>
       <c r="D11" s="7"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="38"/>
-      <c r="G11" s="101"/>
-      <c r="H11" s="102"/>
-      <c r="I11" s="103"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="100"/>
+      <c r="H11" s="101"/>
+      <c r="I11" s="101"/>
       <c r="J11" s="101"/>
-      <c r="K11" s="102"/>
-      <c r="L11" s="103"/>
+      <c r="K11" s="101"/>
+      <c r="L11" s="101"/>
       <c r="M11" s="101"/>
-      <c r="N11" s="102"/>
-      <c r="O11" s="103"/>
-    </row>
-    <row r="12" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N11" s="101"/>
+      <c r="O11" s="102"/>
+      <c r="P11" s="92"/>
+      <c r="Q11" s="93"/>
+      <c r="R11" s="94"/>
+    </row>
+    <row r="12" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="2"/>
       <c r="C12" s="5"/>
       <c r="D12" s="7"/>
-      <c r="E12" s="35" t="s">
+      <c r="E12" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="F12" s="36"/>
-      <c r="G12" s="115" t="s">
-        <v>30</v>
-      </c>
-      <c r="H12" s="116"/>
-      <c r="I12" s="117"/>
-      <c r="J12" s="115" t="s">
-        <v>31</v>
-      </c>
-      <c r="K12" s="116"/>
-      <c r="L12" s="117"/>
-      <c r="M12" s="115" t="s">
-        <v>14</v>
-      </c>
-      <c r="N12" s="116"/>
-      <c r="O12" s="117"/>
-    </row>
-    <row r="13" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F12" s="40"/>
+      <c r="G12" s="113" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" s="114"/>
+      <c r="I12" s="115"/>
+      <c r="J12" s="113" t="s">
+        <v>65</v>
+      </c>
+      <c r="K12" s="114"/>
+      <c r="L12" s="115"/>
+      <c r="M12" s="113" t="s">
+        <v>64</v>
+      </c>
+      <c r="N12" s="114"/>
+      <c r="O12" s="115"/>
+      <c r="P12" s="89" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q12" s="90"/>
+      <c r="R12" s="91"/>
+    </row>
+    <row r="13" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="5"/>
       <c r="D13" s="7"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="118"/>
-      <c r="H13" s="119"/>
-      <c r="I13" s="120"/>
-      <c r="J13" s="118"/>
-      <c r="K13" s="119"/>
-      <c r="L13" s="120"/>
-      <c r="M13" s="118"/>
-      <c r="N13" s="119"/>
-      <c r="O13" s="120"/>
-    </row>
-    <row r="14" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E13" s="39"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="116"/>
+      <c r="H13" s="117"/>
+      <c r="I13" s="118"/>
+      <c r="J13" s="116"/>
+      <c r="K13" s="117"/>
+      <c r="L13" s="118"/>
+      <c r="M13" s="116"/>
+      <c r="N13" s="117"/>
+      <c r="O13" s="118"/>
+      <c r="P13" s="92"/>
+      <c r="Q13" s="93"/>
+      <c r="R13" s="94"/>
+    </row>
+    <row r="14" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="C14" s="5"/>
       <c r="D14" s="7"/>
-      <c r="E14" s="37" t="s">
-        <v>22</v>
-      </c>
-      <c r="F14" s="38"/>
-      <c r="G14" s="121">
-        <f>87*110%</f>
-        <v>95.7</v>
-      </c>
-      <c r="H14" s="122"/>
-      <c r="I14" s="104" t="s">
+      <c r="E14" s="41" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="42"/>
+      <c r="G14" s="103"/>
+      <c r="H14" s="104"/>
+      <c r="I14" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="J14" s="125"/>
-      <c r="K14" s="126"/>
-      <c r="L14" s="104" t="s">
+      <c r="J14" s="103">
+        <f>85*110%</f>
+        <v>93.500000000000014</v>
+      </c>
+      <c r="K14" s="104"/>
+      <c r="L14" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="M14" s="125"/>
-      <c r="N14" s="126"/>
-      <c r="O14" s="104" t="s">
+      <c r="M14" s="103">
+        <f>94*110%</f>
+        <v>103.4</v>
+      </c>
+      <c r="N14" s="104"/>
+      <c r="O14" s="95" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P14" s="103"/>
+      <c r="Q14" s="104"/>
+      <c r="R14" s="95" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="2"/>
       <c r="C15" s="5"/>
       <c r="D15" s="7"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="38"/>
-      <c r="G15" s="123"/>
-      <c r="H15" s="124"/>
-      <c r="I15" s="105"/>
-      <c r="J15" s="127"/>
-      <c r="K15" s="128"/>
-      <c r="L15" s="105"/>
-      <c r="M15" s="127"/>
-      <c r="N15" s="128"/>
-      <c r="O15" s="105"/>
-    </row>
-    <row r="16" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E15" s="41"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="105"/>
+      <c r="H15" s="106"/>
+      <c r="I15" s="96"/>
+      <c r="J15" s="105"/>
+      <c r="K15" s="106"/>
+      <c r="L15" s="96"/>
+      <c r="M15" s="105"/>
+      <c r="N15" s="106"/>
+      <c r="O15" s="96"/>
+      <c r="P15" s="105"/>
+      <c r="Q15" s="106"/>
+      <c r="R15" s="96"/>
+    </row>
+    <row r="16" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="2"/>
       <c r="C16" s="5"/>
       <c r="D16" s="7"/>
-      <c r="E16" s="37" t="s">
+      <c r="E16" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="F16" s="38"/>
-      <c r="G16" s="84">
-        <v>3.0555555555555557E-3</v>
-      </c>
-      <c r="H16" s="85"/>
-      <c r="I16" s="70" t="s">
+      <c r="F16" s="42"/>
+      <c r="G16" s="81">
+        <v>2.662037037037037E-3</v>
+      </c>
+      <c r="H16" s="82"/>
+      <c r="I16" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="J16" s="84"/>
-      <c r="K16" s="85"/>
-      <c r="L16" s="70" t="s">
+      <c r="J16" s="81">
+        <v>2.5231481481481481E-3</v>
+      </c>
+      <c r="K16" s="82"/>
+      <c r="L16" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="M16" s="84"/>
-      <c r="N16" s="85"/>
-      <c r="O16" s="70" t="s">
+      <c r="M16" s="81">
+        <v>3.1712962962962962E-3</v>
+      </c>
+      <c r="N16" s="82"/>
+      <c r="O16" s="31" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="2:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P16" s="128">
+        <v>5.9027777777777776E-3</v>
+      </c>
+      <c r="Q16" s="129"/>
+      <c r="R16" s="87" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="3"/>
       <c r="C17" s="4"/>
       <c r="D17" s="8"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="38"/>
-      <c r="G17" s="86"/>
-      <c r="H17" s="87"/>
-      <c r="I17" s="71"/>
-      <c r="J17" s="86"/>
-      <c r="K17" s="87"/>
-      <c r="L17" s="71"/>
-      <c r="M17" s="86"/>
-      <c r="N17" s="87"/>
-      <c r="O17" s="71"/>
-    </row>
-    <row r="18" spans="2:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="72" t="s">
+      <c r="E17" s="41"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="83"/>
+      <c r="H17" s="84"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="83"/>
+      <c r="K17" s="84"/>
+      <c r="L17" s="32"/>
+      <c r="M17" s="83"/>
+      <c r="N17" s="84"/>
+      <c r="O17" s="32"/>
+      <c r="P17" s="130"/>
+      <c r="Q17" s="131"/>
+      <c r="R17" s="88"/>
+    </row>
+    <row r="18" spans="2:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="73"/>
-      <c r="D18" s="73"/>
-      <c r="E18" s="73"/>
-      <c r="F18" s="73"/>
-      <c r="G18" s="73"/>
-      <c r="H18" s="73"/>
-      <c r="I18" s="73"/>
-      <c r="J18" s="73"/>
-      <c r="K18" s="73"/>
-      <c r="L18" s="73"/>
-      <c r="M18" s="73"/>
-      <c r="N18" s="73"/>
-      <c r="O18" s="74"/>
-    </row>
-    <row r="19" spans="2:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="75"/>
-      <c r="C19" s="76"/>
-      <c r="D19" s="76"/>
-      <c r="E19" s="76"/>
-      <c r="F19" s="76"/>
-      <c r="G19" s="76"/>
-      <c r="H19" s="76"/>
-      <c r="I19" s="76"/>
-      <c r="J19" s="76"/>
-      <c r="K19" s="76"/>
-      <c r="L19" s="76"/>
-      <c r="M19" s="76"/>
-      <c r="N19" s="76"/>
-      <c r="O19" s="77"/>
-    </row>
-    <row r="20" spans="2:15" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="55" t="s">
-        <v>16</v>
-      </c>
-      <c r="C20" s="56"/>
-      <c r="D20" s="56"/>
-      <c r="E20" s="56"/>
-      <c r="F20" s="56"/>
-      <c r="G20" s="58" t="s">
-        <v>25</v>
-      </c>
-      <c r="H20" s="59"/>
-      <c r="I20" s="60"/>
-      <c r="J20" s="58"/>
-      <c r="K20" s="59"/>
-      <c r="L20" s="60"/>
-      <c r="M20" s="58"/>
-      <c r="N20" s="59"/>
-      <c r="O20" s="60"/>
-    </row>
-    <row r="21" spans="2:15" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="41"/>
-      <c r="C21" s="57"/>
-      <c r="D21" s="57"/>
-      <c r="E21" s="57"/>
-      <c r="F21" s="57"/>
-      <c r="G21" s="61"/>
-      <c r="H21" s="62"/>
-      <c r="I21" s="63"/>
-      <c r="J21" s="61"/>
-      <c r="K21" s="62"/>
-      <c r="L21" s="63"/>
-      <c r="M21" s="61"/>
-      <c r="N21" s="62"/>
-      <c r="O21" s="63"/>
-    </row>
-    <row r="22" spans="2:15" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="39" t="s">
+      <c r="C18" s="70"/>
+      <c r="D18" s="70"/>
+      <c r="E18" s="70"/>
+      <c r="F18" s="70"/>
+      <c r="G18" s="70"/>
+      <c r="H18" s="70"/>
+      <c r="I18" s="70"/>
+      <c r="J18" s="70"/>
+      <c r="K18" s="70"/>
+      <c r="L18" s="70"/>
+      <c r="M18" s="70"/>
+      <c r="N18" s="70"/>
+      <c r="O18" s="70"/>
+      <c r="P18" s="70"/>
+      <c r="Q18" s="70"/>
+      <c r="R18" s="71"/>
+    </row>
+    <row r="19" spans="2:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="72"/>
+      <c r="C19" s="73"/>
+      <c r="D19" s="73"/>
+      <c r="E19" s="73"/>
+      <c r="F19" s="73"/>
+      <c r="G19" s="73"/>
+      <c r="H19" s="73"/>
+      <c r="I19" s="73"/>
+      <c r="J19" s="73"/>
+      <c r="K19" s="73"/>
+      <c r="L19" s="73"/>
+      <c r="M19" s="73"/>
+      <c r="N19" s="73"/>
+      <c r="O19" s="73"/>
+      <c r="P19" s="73"/>
+      <c r="Q19" s="73"/>
+      <c r="R19" s="74"/>
+    </row>
+    <row r="20" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="60"/>
+      <c r="D20" s="60"/>
+      <c r="E20" s="60"/>
+      <c r="F20" s="60"/>
+      <c r="G20" s="63" t="s">
+        <v>69</v>
+      </c>
+      <c r="H20" s="64"/>
+      <c r="I20" s="65"/>
+      <c r="J20" s="63" t="s">
+        <v>68</v>
+      </c>
+      <c r="K20" s="64"/>
+      <c r="L20" s="65"/>
+      <c r="M20" s="63" t="s">
+        <v>23</v>
+      </c>
+      <c r="N20" s="64"/>
+      <c r="O20" s="65"/>
+      <c r="P20" s="63" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q20" s="64"/>
+      <c r="R20" s="65"/>
+    </row>
+    <row r="21" spans="2:18" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="61"/>
+      <c r="C21" s="62"/>
+      <c r="D21" s="62"/>
+      <c r="E21" s="62"/>
+      <c r="F21" s="62"/>
+      <c r="G21" s="66"/>
+      <c r="H21" s="67"/>
+      <c r="I21" s="68"/>
+      <c r="J21" s="66"/>
+      <c r="K21" s="67"/>
+      <c r="L21" s="68"/>
+      <c r="M21" s="66"/>
+      <c r="N21" s="67"/>
+      <c r="O21" s="68"/>
+      <c r="P21" s="66"/>
+      <c r="Q21" s="67"/>
+      <c r="R21" s="68"/>
+    </row>
+    <row r="22" spans="2:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="40"/>
-      <c r="D22" s="82" t="s">
+      <c r="C22" s="44"/>
+      <c r="D22" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="82"/>
-      <c r="F22" s="82"/>
-      <c r="G22" s="64" t="s">
+      <c r="E22" s="79"/>
+      <c r="F22" s="79"/>
+      <c r="G22" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="H22" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="I22" s="28"/>
+      <c r="J22" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="K22" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="L22" s="28"/>
+      <c r="M22" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="N22" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="O22" s="28"/>
+      <c r="P22" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q22" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="R22" s="28"/>
+    </row>
+    <row r="23" spans="2:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="45"/>
+      <c r="C23" s="46"/>
+      <c r="D23" s="80"/>
+      <c r="E23" s="80"/>
+      <c r="F23" s="80"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="30"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="29"/>
+      <c r="L23" s="30"/>
+      <c r="M23" s="26"/>
+      <c r="N23" s="29"/>
+      <c r="O23" s="30"/>
+      <c r="P23" s="26"/>
+      <c r="Q23" s="29"/>
+      <c r="R23" s="30"/>
+    </row>
+    <row r="24" spans="2:18" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="47">
+        <v>0.52</v>
+      </c>
+      <c r="C24" s="48"/>
+      <c r="D24" s="51" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" s="52"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="33" t="s">
         <v>17</v>
-      </c>
-      <c r="H22" s="66" t="s">
-        <v>15</v>
-      </c>
-      <c r="I22" s="67"/>
-      <c r="J22" s="64"/>
-      <c r="K22" s="66"/>
-      <c r="L22" s="67"/>
-      <c r="M22" s="64"/>
-      <c r="N22" s="66"/>
-      <c r="O22" s="67"/>
-    </row>
-    <row r="23" spans="2:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="41"/>
-      <c r="C23" s="42"/>
-      <c r="D23" s="83"/>
-      <c r="E23" s="83"/>
-      <c r="F23" s="83"/>
-      <c r="G23" s="65"/>
-      <c r="H23" s="68"/>
-      <c r="I23" s="69"/>
-      <c r="J23" s="65"/>
-      <c r="K23" s="68"/>
-      <c r="L23" s="69"/>
-      <c r="M23" s="65"/>
-      <c r="N23" s="68"/>
-      <c r="O23" s="69"/>
-    </row>
-    <row r="24" spans="2:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="43">
-        <v>0.52</v>
-      </c>
-      <c r="C24" s="44"/>
-      <c r="D24" s="47" t="s">
-        <v>20</v>
-      </c>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="90" t="s">
-        <v>19</v>
       </c>
       <c r="H24" s="27" t="s">
         <v>10</v>
       </c>
       <c r="I24" s="28"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="31"/>
-      <c r="L24" s="32"/>
-      <c r="M24" s="25"/>
-      <c r="N24" s="31"/>
-      <c r="O24" s="32"/>
-    </row>
-    <row r="25" spans="2:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="45"/>
-      <c r="C25" s="46"/>
-      <c r="D25" s="88" t="s">
-        <v>21</v>
-      </c>
-      <c r="E25" s="89"/>
-      <c r="F25" s="89"/>
-      <c r="G25" s="91"/>
+      <c r="J24" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="K24" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="L24" s="28"/>
+      <c r="M24" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="N24" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="O24" s="28"/>
+      <c r="P24" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q24" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="R24" s="28"/>
+    </row>
+    <row r="25" spans="2:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="49"/>
+      <c r="C25" s="50"/>
+      <c r="D25" s="85" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" s="86"/>
+      <c r="F25" s="86"/>
+      <c r="G25" s="34"/>
       <c r="H25" s="29"/>
       <c r="I25" s="30"/>
-      <c r="J25" s="26"/>
-      <c r="K25" s="33"/>
-      <c r="L25" s="34"/>
-      <c r="M25" s="26"/>
-      <c r="N25" s="33"/>
-      <c r="O25" s="34"/>
-    </row>
-    <row r="26" spans="2:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="43">
-        <v>0.01</v>
-      </c>
-      <c r="C26" s="44"/>
-      <c r="D26" s="47" t="s">
-        <v>27</v>
-      </c>
-      <c r="E26" s="48"/>
-      <c r="F26" s="48"/>
-      <c r="G26" s="90" t="s">
-        <v>28</v>
-      </c>
-      <c r="H26" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="I26" s="32"/>
-      <c r="J26" s="25"/>
-      <c r="K26" s="31"/>
-      <c r="L26" s="32"/>
-      <c r="M26" s="25"/>
-      <c r="N26" s="31"/>
-      <c r="O26" s="32"/>
-    </row>
-    <row r="27" spans="2:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="45"/>
-      <c r="C27" s="46"/>
-      <c r="D27" s="88">
-        <v>40</v>
-      </c>
-      <c r="E27" s="89"/>
-      <c r="F27" s="89"/>
-      <c r="G27" s="91"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="34"/>
-      <c r="J27" s="26"/>
-      <c r="K27" s="33"/>
-      <c r="L27" s="34"/>
-      <c r="M27" s="26"/>
-      <c r="N27" s="33"/>
-      <c r="O27" s="34"/>
-    </row>
-    <row r="28" spans="2:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="43">
-        <v>0.47</v>
-      </c>
-      <c r="C28" s="44"/>
-      <c r="D28" s="47" t="s">
-        <v>18</v>
-      </c>
-      <c r="E28" s="48"/>
-      <c r="F28" s="48"/>
-      <c r="G28" s="90" t="s">
-        <v>24</v>
-      </c>
-      <c r="H28" s="31" t="s">
+      <c r="J25" s="34"/>
+      <c r="K25" s="29"/>
+      <c r="L25" s="30"/>
+      <c r="M25" s="34"/>
+      <c r="N25" s="29"/>
+      <c r="O25" s="30"/>
+      <c r="P25" s="34"/>
+      <c r="Q25" s="29"/>
+      <c r="R25" s="30"/>
+    </row>
+    <row r="26" spans="2:18" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="47">
+        <v>0.48</v>
+      </c>
+      <c r="C26" s="48"/>
+      <c r="D26" s="51" t="s">
+        <v>16</v>
+      </c>
+      <c r="E26" s="52"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="33" t="s">
+        <v>70</v>
+      </c>
+      <c r="H26" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="I28" s="32"/>
-      <c r="J28" s="25"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="32"/>
-      <c r="M28" s="25"/>
-      <c r="N28" s="31"/>
-      <c r="O28" s="32"/>
-    </row>
-    <row r="29" spans="2:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="45"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="88" t="s">
+      <c r="I26" s="36"/>
+      <c r="J26" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="K26" s="35" t="s">
+        <v>10</v>
+      </c>
+      <c r="L26" s="36"/>
+      <c r="M26" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="N26" s="35" t="s">
+        <v>10</v>
+      </c>
+      <c r="O26" s="36"/>
+      <c r="P26" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q26" s="35" t="s">
+        <v>10</v>
+      </c>
+      <c r="R26" s="36"/>
+    </row>
+    <row r="27" spans="2:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="49"/>
+      <c r="C27" s="50"/>
+      <c r="D27" s="85" t="s">
         <v>12</v>
       </c>
-      <c r="E29" s="89"/>
-      <c r="F29" s="89"/>
-      <c r="G29" s="91"/>
-      <c r="H29" s="33"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="26"/>
-      <c r="K29" s="33"/>
-      <c r="L29" s="34"/>
-      <c r="M29" s="26"/>
-      <c r="N29" s="33"/>
-      <c r="O29" s="34"/>
-    </row>
-    <row r="30" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="43"/>
-      <c r="C30" s="44"/>
-      <c r="D30" s="47"/>
-      <c r="E30" s="48"/>
-      <c r="F30" s="48"/>
-      <c r="G30" s="90"/>
-      <c r="H30" s="31"/>
-      <c r="I30" s="32"/>
-      <c r="J30" s="25"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="28"/>
-      <c r="M30" s="25"/>
-      <c r="N30" s="27"/>
-      <c r="O30" s="28"/>
-    </row>
-    <row r="31" spans="2:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="45"/>
-      <c r="C31" s="46"/>
-      <c r="D31" s="88"/>
-      <c r="E31" s="89"/>
-      <c r="F31" s="89"/>
-      <c r="G31" s="91"/>
-      <c r="H31" s="33"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="26"/>
-      <c r="K31" s="29"/>
-      <c r="L31" s="30"/>
-      <c r="M31" s="26"/>
-      <c r="N31" s="29"/>
-      <c r="O31" s="30"/>
-    </row>
-    <row r="32" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="E27" s="86"/>
+      <c r="F27" s="86"/>
+      <c r="G27" s="34"/>
+      <c r="H27" s="37"/>
+      <c r="I27" s="38"/>
+      <c r="J27" s="34"/>
+      <c r="K27" s="37"/>
+      <c r="L27" s="38"/>
+      <c r="M27" s="34"/>
+      <c r="N27" s="37"/>
+      <c r="O27" s="38"/>
+      <c r="P27" s="34"/>
+      <c r="Q27" s="37"/>
+      <c r="R27" s="38"/>
+    </row>
+    <row r="28" spans="2:18" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="47"/>
+      <c r="C28" s="48"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="52"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="35"/>
+      <c r="I28" s="36"/>
+      <c r="J28" s="33"/>
+      <c r="K28" s="35"/>
+      <c r="L28" s="36"/>
+      <c r="M28" s="33"/>
+      <c r="N28" s="35"/>
+      <c r="O28" s="36"/>
+      <c r="P28" s="33"/>
+      <c r="Q28" s="35"/>
+      <c r="R28" s="36"/>
+    </row>
+    <row r="29" spans="2:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="49"/>
+      <c r="C29" s="50"/>
+      <c r="D29" s="85"/>
+      <c r="E29" s="86"/>
+      <c r="F29" s="86"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="37"/>
+      <c r="I29" s="38"/>
+      <c r="J29" s="34"/>
+      <c r="K29" s="37"/>
+      <c r="L29" s="38"/>
+      <c r="M29" s="34"/>
+      <c r="N29" s="37"/>
+      <c r="O29" s="38"/>
+      <c r="P29" s="34"/>
+      <c r="Q29" s="37"/>
+      <c r="R29" s="38"/>
+    </row>
+    <row r="30" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2996,47 +3119,42 @@
     <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="78">
-    <mergeCell ref="B30:C31"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H24:I25"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="G30:G31"/>
-    <mergeCell ref="H30:I31"/>
-    <mergeCell ref="D30:F30"/>
+  <mergeCells count="83">
+    <mergeCell ref="J14:K15"/>
+    <mergeCell ref="O14:O15"/>
     <mergeCell ref="B28:C29"/>
     <mergeCell ref="B26:C27"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="E4:O7"/>
+    <mergeCell ref="E4:R7"/>
     <mergeCell ref="J24:J25"/>
     <mergeCell ref="K24:L25"/>
-    <mergeCell ref="M24:M25"/>
-    <mergeCell ref="N24:O25"/>
-    <mergeCell ref="M10:O11"/>
-    <mergeCell ref="M16:N17"/>
-    <mergeCell ref="N22:O23"/>
+    <mergeCell ref="P24:P25"/>
+    <mergeCell ref="Q24:R25"/>
+    <mergeCell ref="P10:R11"/>
+    <mergeCell ref="P16:Q17"/>
+    <mergeCell ref="Q22:R23"/>
     <mergeCell ref="I14:I15"/>
     <mergeCell ref="G20:I21"/>
     <mergeCell ref="G12:I13"/>
     <mergeCell ref="J12:L13"/>
     <mergeCell ref="G14:H15"/>
-    <mergeCell ref="J14:K15"/>
-    <mergeCell ref="M14:N15"/>
-    <mergeCell ref="M12:O13"/>
-    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="P20:R21"/>
+    <mergeCell ref="R16:R17"/>
+    <mergeCell ref="P8:R9"/>
+    <mergeCell ref="R14:R15"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="M16:N17"/>
+    <mergeCell ref="G10:O11"/>
+    <mergeCell ref="O16:O17"/>
     <mergeCell ref="M20:O21"/>
-    <mergeCell ref="O16:O17"/>
-    <mergeCell ref="M8:O9"/>
-    <mergeCell ref="G10:I11"/>
-    <mergeCell ref="J10:L11"/>
-    <mergeCell ref="O14:O15"/>
-    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="P14:Q15"/>
+    <mergeCell ref="P12:R13"/>
     <mergeCell ref="G8:I9"/>
     <mergeCell ref="J8:L9"/>
-    <mergeCell ref="M22:M23"/>
+    <mergeCell ref="M8:O9"/>
+    <mergeCell ref="M12:O13"/>
+    <mergeCell ref="M14:N15"/>
+    <mergeCell ref="P22:P23"/>
     <mergeCell ref="D29:F29"/>
     <mergeCell ref="D26:F26"/>
     <mergeCell ref="G26:G27"/>
@@ -3045,10 +3163,13 @@
     <mergeCell ref="J26:J27"/>
     <mergeCell ref="J28:J29"/>
     <mergeCell ref="K26:L27"/>
-    <mergeCell ref="M26:M27"/>
+    <mergeCell ref="P26:P27"/>
     <mergeCell ref="D28:F28"/>
     <mergeCell ref="G28:G29"/>
     <mergeCell ref="H28:I29"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H24:I25"/>
+    <mergeCell ref="D25:F25"/>
     <mergeCell ref="B2:D3"/>
     <mergeCell ref="B20:F21"/>
     <mergeCell ref="J20:L21"/>
@@ -3057,8 +3178,8 @@
     <mergeCell ref="G22:G23"/>
     <mergeCell ref="H22:I23"/>
     <mergeCell ref="L16:L17"/>
-    <mergeCell ref="B18:O19"/>
-    <mergeCell ref="E2:O3"/>
+    <mergeCell ref="B18:R19"/>
+    <mergeCell ref="E2:R3"/>
     <mergeCell ref="E8:F9"/>
     <mergeCell ref="E10:F11"/>
     <mergeCell ref="D22:F23"/>
@@ -3070,16 +3191,21 @@
     <mergeCell ref="B22:C23"/>
     <mergeCell ref="B24:C25"/>
     <mergeCell ref="D24:F24"/>
-    <mergeCell ref="J30:J31"/>
-    <mergeCell ref="K30:L31"/>
+    <mergeCell ref="Q26:R27"/>
+    <mergeCell ref="K28:L29"/>
+    <mergeCell ref="P28:P29"/>
+    <mergeCell ref="Q28:R29"/>
+    <mergeCell ref="M26:M27"/>
     <mergeCell ref="N26:O27"/>
-    <mergeCell ref="K28:L29"/>
     <mergeCell ref="M28:M29"/>
     <mergeCell ref="N28:O29"/>
-    <mergeCell ref="M30:M31"/>
-    <mergeCell ref="N30:O31"/>
+    <mergeCell ref="M22:M23"/>
+    <mergeCell ref="N22:O23"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="M24:M25"/>
+    <mergeCell ref="N24:O25"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.12" right="0.12" top="0.28999999999999998" bottom="0" header="0.18" footer="0"/>
   <pageSetup scale="115" orientation="landscape" r:id="rId1"/>
@@ -3103,14 +3229,14 @@
   <sheetData>
     <row r="1" spans="1:13" ht="27" x14ac:dyDescent="0.5">
       <c r="B1" s="10" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C1" s="10"/>
       <c r="D1" s="11"/>
     </row>
     <row r="2" spans="1:13" ht="27" x14ac:dyDescent="0.5">
       <c r="A2" s="12" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="10"/>
@@ -3118,7 +3244,7 @@
     </row>
     <row r="3" spans="1:13" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A3" s="9" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -3126,54 +3252,54 @@
     </row>
     <row r="4" spans="1:13" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A4" s="9" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="H4" s="13" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="I4" s="13"/>
       <c r="J4" s="13"/>
     </row>
     <row r="5" spans="1:13" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A5" s="9" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D5" s="9"/>
-      <c r="F5" s="129">
+      <c r="F5" s="132">
         <f>SUM(F7:F22)</f>
         <v>7.05</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="F6" s="130"/>
+      <c r="F6" s="133"/>
       <c r="H6" s="13" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="19" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -3181,7 +3307,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="J7" s="13" t="s">
         <v>12</v>
@@ -3203,10 +3329,10 @@
     </row>
     <row r="9" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A9" s="19" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
@@ -3214,13 +3340,13 @@
         <v>1.2</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="I9" s="21">
         <v>9.5699999999999993E-2</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
@@ -3232,10 +3358,10 @@
     </row>
     <row r="11" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A11" s="19" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -3243,13 +3369,13 @@
         <v>0.5</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="J11" s="23">
         <v>0.21</v>
       </c>
       <c r="K11" s="14" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="M11" s="14"/>
     </row>
@@ -3263,23 +3389,23 @@
         <v>2.3E-2</v>
       </c>
       <c r="K12" s="14" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A13" s="19" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B13" s="20"/>
       <c r="C13" s="12" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D13" s="12"/>
       <c r="F13" s="16">
         <v>0.7</v>
       </c>
       <c r="H13" s="21" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
@@ -3288,27 +3414,27 @@
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
       <c r="F14" s="17"/>
-      <c r="H14" s="131">
+      <c r="H14" s="134">
         <f>J12+I9</f>
         <v>0.1187</v>
       </c>
       <c r="I14" s="18" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A15" s="19" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
       <c r="F15" s="16">
         <v>0.7</v>
       </c>
-      <c r="H15" s="131"/>
+      <c r="H15" s="134"/>
     </row>
     <row r="16" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A16" s="19"/>
@@ -3319,10 +3445,10 @@
     </row>
     <row r="17" spans="1:6" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A17" s="19" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
@@ -3339,10 +3465,10 @@
     </row>
     <row r="19" spans="1:6" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A19" s="19" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
@@ -3353,7 +3479,7 @@
     <row r="20" spans="1:6" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A20" s="19"/>
       <c r="B20" s="20" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
@@ -3370,11 +3496,11 @@
     </row>
     <row r="22" spans="1:6" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A22" s="12" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="12" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D22" s="12"/>
       <c r="F22" s="16">

</xml_diff>

<commit_message>
Sincronizaci├│n autom├ítica 02/02/2026 11:06:02.07
</commit_message>
<xml_diff>
--- a/Fichas/Q037.xlsx
+++ b/Fichas/Q037.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\DESKTOP-ID9UEKK\Users\Admin\Desktop\CONTROL DISEÑO\VIVA ROUSS\QPTIMA 2025\DESAROLLOS 25\Q037 CROP TOP TEEN CON CINTAS EN LA SIZA Y CUELLO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Programacion\MAES2O26\Fichas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DCA8930-9CD0-4113-AA53-A5F1A3B7E081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F4C5573-B290-448D-A83F-BA659713F46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FICHA TECNICA" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="74">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -250,7 +250,13 @@
     <t>#7</t>
   </si>
   <si>
-    <t>MAQ#31</t>
+    <t>MAQ</t>
+  </si>
+  <si>
+    <t>#01</t>
+  </si>
+  <si>
+    <t>#31</t>
   </si>
 </sst>
 </file>
@@ -454,13 +460,6 @@
     </font>
     <font>
       <b/>
-      <sz val="26"/>
-      <color rgb="FF000000"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <b/>
       <sz val="8"/>
       <name val="Consolas"/>
       <family val="3"/>
@@ -496,6 +495,13 @@
       <b/>
       <sz val="8"/>
       <color theme="0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color rgb="FF000000"/>
       <name val="Consolas"/>
       <family val="3"/>
     </font>
@@ -768,7 +774,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="135">
+  <cellXfs count="140">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -824,34 +830,196 @@
     <xf numFmtId="20" fontId="22" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="26" fillId="7" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="26" fillId="7" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="26" fillId="7" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="26" fillId="7" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="28" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="28" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="28" fillId="10" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="28" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="35" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="35" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="7" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="7" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="30" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="30" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="31" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="31" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -866,48 +1034,6 @@
     <xf numFmtId="49" fontId="8" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="26" fillId="7" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="26" fillId="7" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="26" fillId="7" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="26" fillId="7" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="28" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -936,24 +1062,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -986,163 +1094,34 @@
     <xf numFmtId="0" fontId="27" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="45" fontId="7" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="7" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="36" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="36" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="28" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="28" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="28" fillId="10" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="28" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1153,6 +1132,48 @@
     </xf>
     <xf numFmtId="165" fontId="21" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1261,7 +1282,7 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>657226</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>24149</xdr:rowOff>
+      <xdr:rowOff>52724</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1697,297 +1718,307 @@
       <c r="R1" s="1"/>
     </row>
     <row r="2" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="75" t="s">
+      <c r="C2" s="94"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="109" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="75"/>
-      <c r="G2" s="75"/>
-      <c r="H2" s="75"/>
-      <c r="I2" s="75"/>
-      <c r="J2" s="75"/>
-      <c r="K2" s="75"/>
-      <c r="L2" s="75"/>
-      <c r="M2" s="75"/>
-      <c r="N2" s="75"/>
-      <c r="O2" s="75"/>
-      <c r="P2" s="75"/>
-      <c r="Q2" s="75"/>
-      <c r="R2" s="76"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="109"/>
+      <c r="J2" s="109"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="109"/>
+      <c r="M2" s="109"/>
+      <c r="N2" s="109"/>
+      <c r="O2" s="109"/>
+      <c r="P2" s="109"/>
+      <c r="Q2" s="109"/>
+      <c r="R2" s="110"/>
     </row>
     <row r="3" spans="1:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="56"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="77"/>
-      <c r="F3" s="77"/>
-      <c r="G3" s="77"/>
-      <c r="H3" s="77"/>
-      <c r="I3" s="77"/>
-      <c r="J3" s="77"/>
-      <c r="K3" s="77"/>
-      <c r="L3" s="77"/>
-      <c r="M3" s="77"/>
-      <c r="N3" s="77"/>
-      <c r="O3" s="77"/>
-      <c r="P3" s="77"/>
-      <c r="Q3" s="77"/>
-      <c r="R3" s="78"/>
-    </row>
-    <row r="4" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="96"/>
+      <c r="C3" s="97"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="111"/>
+      <c r="F3" s="111"/>
+      <c r="G3" s="111"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="111"/>
+      <c r="L3" s="111"/>
+      <c r="M3" s="111"/>
+      <c r="N3" s="111"/>
+      <c r="O3" s="111"/>
+      <c r="P3" s="111"/>
+      <c r="Q3" s="111"/>
+      <c r="R3" s="112"/>
+    </row>
+    <row r="4" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
-      <c r="E4" s="119" t="s">
+      <c r="E4" s="129" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="120"/>
-      <c r="G4" s="120"/>
-      <c r="H4" s="120"/>
-      <c r="I4" s="120"/>
-      <c r="J4" s="120"/>
-      <c r="K4" s="120"/>
-      <c r="L4" s="120"/>
-      <c r="M4" s="120"/>
-      <c r="N4" s="120"/>
-      <c r="O4" s="120"/>
-      <c r="P4" s="120"/>
-      <c r="Q4" s="120"/>
-      <c r="R4" s="121"/>
-    </row>
-    <row r="5" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F4" s="130"/>
+      <c r="G4" s="130"/>
+      <c r="H4" s="130"/>
+      <c r="I4" s="130"/>
+      <c r="J4" s="130"/>
+      <c r="K4" s="130"/>
+      <c r="L4" s="130"/>
+      <c r="M4" s="130"/>
+      <c r="N4" s="130"/>
+      <c r="O4" s="130"/>
+      <c r="P4" s="130"/>
+      <c r="Q4" s="130"/>
+      <c r="R4" s="131"/>
+    </row>
+    <row r="5" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
       <c r="C5" s="5"/>
       <c r="D5" s="7"/>
-      <c r="E5" s="122"/>
-      <c r="F5" s="123"/>
-      <c r="G5" s="123"/>
-      <c r="H5" s="123"/>
-      <c r="I5" s="123"/>
-      <c r="J5" s="123"/>
-      <c r="K5" s="123"/>
-      <c r="L5" s="123"/>
-      <c r="M5" s="123"/>
-      <c r="N5" s="123"/>
-      <c r="O5" s="123"/>
-      <c r="P5" s="123"/>
-      <c r="Q5" s="123"/>
-      <c r="R5" s="124"/>
-    </row>
-    <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E5" s="132"/>
+      <c r="F5" s="133"/>
+      <c r="G5" s="133"/>
+      <c r="H5" s="133"/>
+      <c r="I5" s="133"/>
+      <c r="J5" s="133"/>
+      <c r="K5" s="133"/>
+      <c r="L5" s="133"/>
+      <c r="M5" s="133"/>
+      <c r="N5" s="133"/>
+      <c r="O5" s="133"/>
+      <c r="P5" s="133"/>
+      <c r="Q5" s="133"/>
+      <c r="R5" s="134"/>
+    </row>
+    <row r="6" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2"/>
       <c r="C6" s="5"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="122"/>
-      <c r="F6" s="123"/>
-      <c r="G6" s="123"/>
-      <c r="H6" s="123"/>
-      <c r="I6" s="123"/>
-      <c r="J6" s="123"/>
-      <c r="K6" s="123"/>
-      <c r="L6" s="123"/>
-      <c r="M6" s="123"/>
-      <c r="N6" s="123"/>
-      <c r="O6" s="123"/>
-      <c r="P6" s="123"/>
-      <c r="Q6" s="123"/>
-      <c r="R6" s="124"/>
-    </row>
-    <row r="7" spans="1:18" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E6" s="132"/>
+      <c r="F6" s="133"/>
+      <c r="G6" s="133"/>
+      <c r="H6" s="133"/>
+      <c r="I6" s="133"/>
+      <c r="J6" s="133"/>
+      <c r="K6" s="133"/>
+      <c r="L6" s="133"/>
+      <c r="M6" s="133"/>
+      <c r="N6" s="133"/>
+      <c r="O6" s="133"/>
+      <c r="P6" s="133"/>
+      <c r="Q6" s="133"/>
+      <c r="R6" s="134"/>
+    </row>
+    <row r="7" spans="1:18" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2"/>
       <c r="C7" s="5"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="125"/>
-      <c r="F7" s="126"/>
-      <c r="G7" s="126"/>
-      <c r="H7" s="126"/>
-      <c r="I7" s="126"/>
-      <c r="J7" s="126"/>
-      <c r="K7" s="126"/>
-      <c r="L7" s="126"/>
-      <c r="M7" s="126"/>
-      <c r="N7" s="126"/>
-      <c r="O7" s="126"/>
-      <c r="P7" s="126"/>
-      <c r="Q7" s="126"/>
-      <c r="R7" s="127"/>
+      <c r="E7" s="135"/>
+      <c r="F7" s="136"/>
+      <c r="G7" s="136"/>
+      <c r="H7" s="136"/>
+      <c r="I7" s="136"/>
+      <c r="J7" s="136"/>
+      <c r="K7" s="136"/>
+      <c r="L7" s="136"/>
+      <c r="M7" s="136"/>
+      <c r="N7" s="136"/>
+      <c r="O7" s="136"/>
+      <c r="P7" s="136"/>
+      <c r="Q7" s="136"/>
+      <c r="R7" s="137"/>
     </row>
     <row r="8" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2"/>
       <c r="C8" s="5"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="41" t="s">
+      <c r="E8" s="113" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="107" t="s">
+      <c r="F8" s="114"/>
+      <c r="G8" s="77" t="s">
         <v>62</v>
       </c>
-      <c r="H8" s="108"/>
-      <c r="I8" s="109"/>
-      <c r="J8" s="107" t="s">
+      <c r="H8" s="78"/>
+      <c r="I8" s="79"/>
+      <c r="J8" s="77" t="s">
         <v>63</v>
       </c>
-      <c r="K8" s="108"/>
-      <c r="L8" s="109"/>
-      <c r="M8" s="107" t="s">
+      <c r="K8" s="78"/>
+      <c r="L8" s="79"/>
+      <c r="M8" s="77" t="s">
         <v>61</v>
       </c>
-      <c r="N8" s="108"/>
-      <c r="O8" s="109"/>
-      <c r="P8" s="89" t="s">
+      <c r="N8" s="78"/>
+      <c r="O8" s="79"/>
+      <c r="P8" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="Q8" s="90"/>
-      <c r="R8" s="91"/>
+      <c r="Q8" s="42"/>
+      <c r="R8" s="43"/>
     </row>
     <row r="9" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2"/>
       <c r="C9" s="5"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="41"/>
-      <c r="F9" s="42"/>
-      <c r="G9" s="110"/>
-      <c r="H9" s="111"/>
-      <c r="I9" s="112"/>
-      <c r="J9" s="110"/>
-      <c r="K9" s="111"/>
-      <c r="L9" s="112"/>
-      <c r="M9" s="110"/>
-      <c r="N9" s="111"/>
-      <c r="O9" s="112"/>
-      <c r="P9" s="92"/>
-      <c r="Q9" s="93"/>
-      <c r="R9" s="94"/>
-    </row>
-    <row r="10" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E9" s="113"/>
+      <c r="F9" s="114"/>
+      <c r="G9" s="80"/>
+      <c r="H9" s="81"/>
+      <c r="I9" s="82"/>
+      <c r="J9" s="80"/>
+      <c r="K9" s="81"/>
+      <c r="L9" s="82"/>
+      <c r="M9" s="80"/>
+      <c r="N9" s="81"/>
+      <c r="O9" s="82"/>
+      <c r="P9" s="44"/>
+      <c r="Q9" s="45"/>
+      <c r="R9" s="46"/>
+    </row>
+    <row r="10" spans="1:18" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2"/>
       <c r="C10" s="5"/>
       <c r="D10" s="7"/>
-      <c r="E10" s="41" t="s">
+      <c r="E10" s="113" t="s">
         <v>3</v>
       </c>
-      <c r="F10" s="42"/>
-      <c r="G10" s="97" t="s">
+      <c r="F10" s="114"/>
+      <c r="G10" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="H10" s="98"/>
-      <c r="I10" s="98"/>
-      <c r="J10" s="98"/>
-      <c r="K10" s="98"/>
-      <c r="L10" s="98"/>
-      <c r="M10" s="98"/>
-      <c r="N10" s="98"/>
-      <c r="O10" s="99"/>
-      <c r="P10" s="89" t="s">
+      <c r="H10" s="70"/>
+      <c r="I10" s="70"/>
+      <c r="J10" s="70"/>
+      <c r="K10" s="70"/>
+      <c r="L10" s="70"/>
+      <c r="M10" s="70"/>
+      <c r="N10" s="70"/>
+      <c r="O10" s="71"/>
+      <c r="P10" s="138" t="s">
         <v>71</v>
       </c>
-      <c r="Q10" s="90"/>
-      <c r="R10" s="91"/>
-    </row>
-    <row r="11" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q10" s="126" t="s">
+        <v>72</v>
+      </c>
+      <c r="R10" s="127"/>
+    </row>
+    <row r="11" spans="1:18" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2"/>
       <c r="C11" s="5"/>
       <c r="D11" s="7"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="100"/>
-      <c r="H11" s="101"/>
-      <c r="I11" s="101"/>
-      <c r="J11" s="101"/>
-      <c r="K11" s="101"/>
-      <c r="L11" s="101"/>
-      <c r="M11" s="101"/>
-      <c r="N11" s="101"/>
-      <c r="O11" s="102"/>
-      <c r="P11" s="92"/>
-      <c r="Q11" s="93"/>
-      <c r="R11" s="94"/>
+      <c r="E11" s="113"/>
+      <c r="F11" s="114"/>
+      <c r="G11" s="72"/>
+      <c r="H11" s="73"/>
+      <c r="I11" s="73"/>
+      <c r="J11" s="73"/>
+      <c r="K11" s="73"/>
+      <c r="L11" s="73"/>
+      <c r="M11" s="73"/>
+      <c r="N11" s="73"/>
+      <c r="O11" s="74"/>
+      <c r="P11" s="139"/>
+      <c r="Q11" s="102" t="s">
+        <v>73</v>
+      </c>
+      <c r="R11" s="128"/>
     </row>
     <row r="12" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="2"/>
       <c r="C12" s="5"/>
       <c r="D12" s="7"/>
-      <c r="E12" s="39" t="s">
+      <c r="E12" s="117" t="s">
         <v>5</v>
       </c>
-      <c r="F12" s="40"/>
-      <c r="G12" s="113" t="s">
+      <c r="F12" s="118"/>
+      <c r="G12" s="57" t="s">
         <v>66</v>
       </c>
-      <c r="H12" s="114"/>
-      <c r="I12" s="115"/>
-      <c r="J12" s="113" t="s">
+      <c r="H12" s="58"/>
+      <c r="I12" s="59"/>
+      <c r="J12" s="57" t="s">
         <v>65</v>
       </c>
-      <c r="K12" s="114"/>
-      <c r="L12" s="115"/>
-      <c r="M12" s="113" t="s">
+      <c r="K12" s="58"/>
+      <c r="L12" s="59"/>
+      <c r="M12" s="57" t="s">
         <v>64</v>
       </c>
-      <c r="N12" s="114"/>
-      <c r="O12" s="115"/>
-      <c r="P12" s="89" t="s">
+      <c r="N12" s="58"/>
+      <c r="O12" s="59"/>
+      <c r="P12" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="Q12" s="90"/>
-      <c r="R12" s="91"/>
+      <c r="Q12" s="42"/>
+      <c r="R12" s="43"/>
     </row>
     <row r="13" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="5"/>
       <c r="D13" s="7"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="116"/>
-      <c r="H13" s="117"/>
-      <c r="I13" s="118"/>
-      <c r="J13" s="116"/>
-      <c r="K13" s="117"/>
-      <c r="L13" s="118"/>
-      <c r="M13" s="116"/>
-      <c r="N13" s="117"/>
-      <c r="O13" s="118"/>
-      <c r="P13" s="92"/>
-      <c r="Q13" s="93"/>
-      <c r="R13" s="94"/>
+      <c r="E13" s="117"/>
+      <c r="F13" s="118"/>
+      <c r="G13" s="60"/>
+      <c r="H13" s="61"/>
+      <c r="I13" s="62"/>
+      <c r="J13" s="60"/>
+      <c r="K13" s="61"/>
+      <c r="L13" s="62"/>
+      <c r="M13" s="60"/>
+      <c r="N13" s="61"/>
+      <c r="O13" s="62"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="45"/>
+      <c r="R13" s="46"/>
     </row>
     <row r="14" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="C14" s="5"/>
       <c r="D14" s="7"/>
-      <c r="E14" s="41" t="s">
+      <c r="E14" s="113" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="42"/>
-      <c r="G14" s="103"/>
-      <c r="H14" s="104"/>
-      <c r="I14" s="95" t="s">
+      <c r="F14" s="114"/>
+      <c r="G14" s="25">
+        <f>71*110%</f>
+        <v>78.100000000000009</v>
+      </c>
+      <c r="H14" s="26"/>
+      <c r="I14" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="J14" s="103">
-        <f>85*110%</f>
-        <v>93.500000000000014</v>
-      </c>
-      <c r="K14" s="104"/>
-      <c r="L14" s="95" t="s">
+      <c r="J14" s="25">
+        <f>80*110%</f>
+        <v>88</v>
+      </c>
+      <c r="K14" s="26"/>
+      <c r="L14" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="M14" s="103">
-        <f>94*110%</f>
-        <v>103.4</v>
-      </c>
-      <c r="N14" s="104"/>
-      <c r="O14" s="95" t="s">
+      <c r="M14" s="25">
+        <f>88*110%</f>
+        <v>96.800000000000011</v>
+      </c>
+      <c r="N14" s="26"/>
+      <c r="O14" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="P14" s="103"/>
-      <c r="Q14" s="104"/>
-      <c r="R14" s="95" t="s">
+      <c r="P14" s="25">
+        <f>181*110%</f>
+        <v>199.10000000000002</v>
+      </c>
+      <c r="Q14" s="26"/>
+      <c r="R14" s="29" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1995,55 +2026,55 @@
       <c r="B15" s="2"/>
       <c r="C15" s="5"/>
       <c r="D15" s="7"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="105"/>
-      <c r="H15" s="106"/>
-      <c r="I15" s="96"/>
-      <c r="J15" s="105"/>
-      <c r="K15" s="106"/>
-      <c r="L15" s="96"/>
-      <c r="M15" s="105"/>
-      <c r="N15" s="106"/>
-      <c r="O15" s="96"/>
-      <c r="P15" s="105"/>
-      <c r="Q15" s="106"/>
-      <c r="R15" s="96"/>
+      <c r="E15" s="113"/>
+      <c r="F15" s="114"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="28"/>
+      <c r="L15" s="30"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="28"/>
+      <c r="O15" s="30"/>
+      <c r="P15" s="27"/>
+      <c r="Q15" s="28"/>
+      <c r="R15" s="30"/>
     </row>
     <row r="16" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="2"/>
       <c r="C16" s="5"/>
       <c r="D16" s="7"/>
-      <c r="E16" s="41" t="s">
+      <c r="E16" s="113" t="s">
         <v>7</v>
       </c>
-      <c r="F16" s="42"/>
-      <c r="G16" s="81">
+      <c r="F16" s="114"/>
+      <c r="G16" s="65">
         <v>2.662037037037037E-3</v>
       </c>
-      <c r="H16" s="82"/>
-      <c r="I16" s="31" t="s">
+      <c r="H16" s="66"/>
+      <c r="I16" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="J16" s="81">
+      <c r="J16" s="65">
         <v>2.5231481481481481E-3</v>
       </c>
-      <c r="K16" s="82"/>
-      <c r="L16" s="31" t="s">
+      <c r="K16" s="66"/>
+      <c r="L16" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="M16" s="81">
+      <c r="M16" s="65">
         <v>3.1712962962962962E-3</v>
       </c>
-      <c r="N16" s="82"/>
-      <c r="O16" s="31" t="s">
+      <c r="N16" s="66"/>
+      <c r="O16" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="P16" s="128">
+      <c r="P16" s="47">
         <v>5.9027777777777776E-3</v>
       </c>
-      <c r="Q16" s="129"/>
-      <c r="R16" s="87" t="s">
+      <c r="Q16" s="48"/>
+      <c r="R16" s="63" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2051,324 +2082,324 @@
       <c r="B17" s="3"/>
       <c r="C17" s="4"/>
       <c r="D17" s="8"/>
-      <c r="E17" s="41"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="83"/>
-      <c r="H17" s="84"/>
-      <c r="I17" s="32"/>
-      <c r="J17" s="83"/>
-      <c r="K17" s="84"/>
-      <c r="L17" s="32"/>
-      <c r="M17" s="83"/>
-      <c r="N17" s="84"/>
-      <c r="O17" s="32"/>
-      <c r="P17" s="130"/>
-      <c r="Q17" s="131"/>
-      <c r="R17" s="88"/>
+      <c r="E17" s="113"/>
+      <c r="F17" s="114"/>
+      <c r="G17" s="67"/>
+      <c r="H17" s="68"/>
+      <c r="I17" s="76"/>
+      <c r="J17" s="67"/>
+      <c r="K17" s="68"/>
+      <c r="L17" s="76"/>
+      <c r="M17" s="67"/>
+      <c r="N17" s="68"/>
+      <c r="O17" s="76"/>
+      <c r="P17" s="49"/>
+      <c r="Q17" s="50"/>
+      <c r="R17" s="64"/>
     </row>
     <row r="18" spans="2:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="69" t="s">
+      <c r="B18" s="103" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="70"/>
-      <c r="D18" s="70"/>
-      <c r="E18" s="70"/>
-      <c r="F18" s="70"/>
-      <c r="G18" s="70"/>
-      <c r="H18" s="70"/>
-      <c r="I18" s="70"/>
-      <c r="J18" s="70"/>
-      <c r="K18" s="70"/>
-      <c r="L18" s="70"/>
-      <c r="M18" s="70"/>
-      <c r="N18" s="70"/>
-      <c r="O18" s="70"/>
-      <c r="P18" s="70"/>
-      <c r="Q18" s="70"/>
-      <c r="R18" s="71"/>
+      <c r="C18" s="104"/>
+      <c r="D18" s="104"/>
+      <c r="E18" s="104"/>
+      <c r="F18" s="104"/>
+      <c r="G18" s="104"/>
+      <c r="H18" s="104"/>
+      <c r="I18" s="104"/>
+      <c r="J18" s="104"/>
+      <c r="K18" s="104"/>
+      <c r="L18" s="104"/>
+      <c r="M18" s="104"/>
+      <c r="N18" s="104"/>
+      <c r="O18" s="104"/>
+      <c r="P18" s="104"/>
+      <c r="Q18" s="104"/>
+      <c r="R18" s="105"/>
     </row>
     <row r="19" spans="2:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="72"/>
-      <c r="C19" s="73"/>
-      <c r="D19" s="73"/>
-      <c r="E19" s="73"/>
-      <c r="F19" s="73"/>
-      <c r="G19" s="73"/>
-      <c r="H19" s="73"/>
-      <c r="I19" s="73"/>
-      <c r="J19" s="73"/>
-      <c r="K19" s="73"/>
-      <c r="L19" s="73"/>
-      <c r="M19" s="73"/>
-      <c r="N19" s="73"/>
-      <c r="O19" s="73"/>
-      <c r="P19" s="73"/>
-      <c r="Q19" s="73"/>
-      <c r="R19" s="74"/>
+      <c r="B19" s="106"/>
+      <c r="C19" s="107"/>
+      <c r="D19" s="107"/>
+      <c r="E19" s="107"/>
+      <c r="F19" s="107"/>
+      <c r="G19" s="107"/>
+      <c r="H19" s="107"/>
+      <c r="I19" s="107"/>
+      <c r="J19" s="107"/>
+      <c r="K19" s="107"/>
+      <c r="L19" s="107"/>
+      <c r="M19" s="107"/>
+      <c r="N19" s="107"/>
+      <c r="O19" s="107"/>
+      <c r="P19" s="107"/>
+      <c r="Q19" s="107"/>
+      <c r="R19" s="108"/>
     </row>
     <row r="20" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="59" t="s">
+      <c r="B20" s="99" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="60"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="63" t="s">
+      <c r="C20" s="100"/>
+      <c r="D20" s="100"/>
+      <c r="E20" s="100"/>
+      <c r="F20" s="100"/>
+      <c r="G20" s="51" t="s">
         <v>69</v>
       </c>
-      <c r="H20" s="64"/>
-      <c r="I20" s="65"/>
-      <c r="J20" s="63" t="s">
+      <c r="H20" s="52"/>
+      <c r="I20" s="53"/>
+      <c r="J20" s="51" t="s">
         <v>68</v>
       </c>
-      <c r="K20" s="64"/>
-      <c r="L20" s="65"/>
-      <c r="M20" s="63" t="s">
+      <c r="K20" s="52"/>
+      <c r="L20" s="53"/>
+      <c r="M20" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="N20" s="64"/>
-      <c r="O20" s="65"/>
-      <c r="P20" s="63" t="s">
+      <c r="N20" s="52"/>
+      <c r="O20" s="53"/>
+      <c r="P20" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="Q20" s="64"/>
-      <c r="R20" s="65"/>
+      <c r="Q20" s="52"/>
+      <c r="R20" s="53"/>
     </row>
     <row r="21" spans="2:18" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="61"/>
-      <c r="C21" s="62"/>
-      <c r="D21" s="62"/>
-      <c r="E21" s="62"/>
-      <c r="F21" s="62"/>
-      <c r="G21" s="66"/>
-      <c r="H21" s="67"/>
-      <c r="I21" s="68"/>
-      <c r="J21" s="66"/>
-      <c r="K21" s="67"/>
-      <c r="L21" s="68"/>
-      <c r="M21" s="66"/>
-      <c r="N21" s="67"/>
-      <c r="O21" s="68"/>
-      <c r="P21" s="66"/>
-      <c r="Q21" s="67"/>
-      <c r="R21" s="68"/>
+      <c r="B21" s="101"/>
+      <c r="C21" s="102"/>
+      <c r="D21" s="102"/>
+      <c r="E21" s="102"/>
+      <c r="F21" s="102"/>
+      <c r="G21" s="54"/>
+      <c r="H21" s="55"/>
+      <c r="I21" s="56"/>
+      <c r="J21" s="54"/>
+      <c r="K21" s="55"/>
+      <c r="L21" s="56"/>
+      <c r="M21" s="54"/>
+      <c r="N21" s="55"/>
+      <c r="O21" s="56"/>
+      <c r="P21" s="54"/>
+      <c r="Q21" s="55"/>
+      <c r="R21" s="56"/>
     </row>
     <row r="22" spans="2:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="43" t="s">
+      <c r="B22" s="119" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="44"/>
-      <c r="D22" s="79" t="s">
+      <c r="C22" s="120"/>
+      <c r="D22" s="115" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="79"/>
-      <c r="F22" s="79"/>
-      <c r="G22" s="25" t="s">
+      <c r="E22" s="115"/>
+      <c r="F22" s="115"/>
+      <c r="G22" s="83" t="s">
         <v>67</v>
       </c>
-      <c r="H22" s="27" t="s">
+      <c r="H22" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="I22" s="28"/>
-      <c r="J22" s="25" t="s">
+      <c r="I22" s="38"/>
+      <c r="J22" s="83" t="s">
         <v>67</v>
       </c>
-      <c r="K22" s="27" t="s">
+      <c r="K22" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="L22" s="28"/>
-      <c r="M22" s="25" t="s">
+      <c r="L22" s="38"/>
+      <c r="M22" s="83" t="s">
         <v>67</v>
       </c>
-      <c r="N22" s="27" t="s">
+      <c r="N22" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="O22" s="28"/>
-      <c r="P22" s="25" t="s">
+      <c r="O22" s="38"/>
+      <c r="P22" s="83" t="s">
         <v>67</v>
       </c>
-      <c r="Q22" s="27" t="s">
+      <c r="Q22" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="R22" s="28"/>
+      <c r="R22" s="38"/>
     </row>
     <row r="23" spans="2:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="45"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="80"/>
-      <c r="E23" s="80"/>
-      <c r="F23" s="80"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="29"/>
-      <c r="I23" s="30"/>
-      <c r="J23" s="26"/>
-      <c r="K23" s="29"/>
-      <c r="L23" s="30"/>
-      <c r="M23" s="26"/>
-      <c r="N23" s="29"/>
-      <c r="O23" s="30"/>
-      <c r="P23" s="26"/>
-      <c r="Q23" s="29"/>
-      <c r="R23" s="30"/>
+      <c r="B23" s="121"/>
+      <c r="C23" s="122"/>
+      <c r="D23" s="116"/>
+      <c r="E23" s="116"/>
+      <c r="F23" s="116"/>
+      <c r="G23" s="84"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="40"/>
+      <c r="J23" s="84"/>
+      <c r="K23" s="39"/>
+      <c r="L23" s="40"/>
+      <c r="M23" s="84"/>
+      <c r="N23" s="39"/>
+      <c r="O23" s="40"/>
+      <c r="P23" s="84"/>
+      <c r="Q23" s="39"/>
+      <c r="R23" s="40"/>
     </row>
     <row r="24" spans="2:18" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="47">
+      <c r="B24" s="31">
         <v>0.52</v>
       </c>
-      <c r="C24" s="48"/>
-      <c r="D24" s="51" t="s">
+      <c r="C24" s="32"/>
+      <c r="D24" s="87" t="s">
         <v>18</v>
       </c>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
-      <c r="G24" s="33" t="s">
+      <c r="E24" s="88"/>
+      <c r="F24" s="88"/>
+      <c r="G24" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="H24" s="27" t="s">
+      <c r="H24" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="I24" s="28"/>
-      <c r="J24" s="33" t="s">
+      <c r="I24" s="38"/>
+      <c r="J24" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="K24" s="27" t="s">
+      <c r="K24" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="L24" s="28"/>
-      <c r="M24" s="33" t="s">
+      <c r="L24" s="38"/>
+      <c r="M24" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="N24" s="27" t="s">
+      <c r="N24" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="O24" s="28"/>
-      <c r="P24" s="33" t="s">
+      <c r="O24" s="38"/>
+      <c r="P24" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="Q24" s="27" t="s">
+      <c r="Q24" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="R24" s="28"/>
+      <c r="R24" s="38"/>
     </row>
     <row r="25" spans="2:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="49"/>
-      <c r="C25" s="50"/>
+      <c r="B25" s="33"/>
+      <c r="C25" s="34"/>
       <c r="D25" s="85" t="s">
         <v>19</v>
       </c>
       <c r="E25" s="86"/>
       <c r="F25" s="86"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="29"/>
-      <c r="I25" s="30"/>
-      <c r="J25" s="34"/>
-      <c r="K25" s="29"/>
-      <c r="L25" s="30"/>
-      <c r="M25" s="34"/>
-      <c r="N25" s="29"/>
-      <c r="O25" s="30"/>
-      <c r="P25" s="34"/>
-      <c r="Q25" s="29"/>
-      <c r="R25" s="30"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="39"/>
+      <c r="I25" s="40"/>
+      <c r="J25" s="36"/>
+      <c r="K25" s="39"/>
+      <c r="L25" s="40"/>
+      <c r="M25" s="36"/>
+      <c r="N25" s="39"/>
+      <c r="O25" s="40"/>
+      <c r="P25" s="36"/>
+      <c r="Q25" s="39"/>
+      <c r="R25" s="40"/>
     </row>
     <row r="26" spans="2:18" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="47">
+      <c r="B26" s="31">
         <v>0.48</v>
       </c>
-      <c r="C26" s="48"/>
-      <c r="D26" s="51" t="s">
+      <c r="C26" s="32"/>
+      <c r="D26" s="87" t="s">
         <v>16</v>
       </c>
-      <c r="E26" s="52"/>
-      <c r="F26" s="52"/>
-      <c r="G26" s="33" t="s">
+      <c r="E26" s="88"/>
+      <c r="F26" s="88"/>
+      <c r="G26" s="35" t="s">
         <v>70</v>
       </c>
-      <c r="H26" s="35" t="s">
+      <c r="H26" s="89" t="s">
         <v>10</v>
       </c>
-      <c r="I26" s="36"/>
-      <c r="J26" s="33" t="s">
+      <c r="I26" s="90"/>
+      <c r="J26" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="K26" s="35" t="s">
+      <c r="K26" s="89" t="s">
         <v>10</v>
       </c>
-      <c r="L26" s="36"/>
-      <c r="M26" s="33" t="s">
+      <c r="L26" s="90"/>
+      <c r="M26" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="N26" s="35" t="s">
+      <c r="N26" s="89" t="s">
         <v>10</v>
       </c>
-      <c r="O26" s="36"/>
-      <c r="P26" s="33" t="s">
+      <c r="O26" s="90"/>
+      <c r="P26" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="Q26" s="35" t="s">
+      <c r="Q26" s="89" t="s">
         <v>10</v>
       </c>
-      <c r="R26" s="36"/>
+      <c r="R26" s="90"/>
     </row>
     <row r="27" spans="2:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="49"/>
-      <c r="C27" s="50"/>
+      <c r="B27" s="33"/>
+      <c r="C27" s="34"/>
       <c r="D27" s="85" t="s">
         <v>12</v>
       </c>
       <c r="E27" s="86"/>
       <c r="F27" s="86"/>
-      <c r="G27" s="34"/>
-      <c r="H27" s="37"/>
-      <c r="I27" s="38"/>
-      <c r="J27" s="34"/>
-      <c r="K27" s="37"/>
-      <c r="L27" s="38"/>
-      <c r="M27" s="34"/>
-      <c r="N27" s="37"/>
-      <c r="O27" s="38"/>
-      <c r="P27" s="34"/>
-      <c r="Q27" s="37"/>
-      <c r="R27" s="38"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="91"/>
+      <c r="I27" s="92"/>
+      <c r="J27" s="36"/>
+      <c r="K27" s="91"/>
+      <c r="L27" s="92"/>
+      <c r="M27" s="36"/>
+      <c r="N27" s="91"/>
+      <c r="O27" s="92"/>
+      <c r="P27" s="36"/>
+      <c r="Q27" s="91"/>
+      <c r="R27" s="92"/>
     </row>
     <row r="28" spans="2:18" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="47"/>
-      <c r="C28" s="48"/>
-      <c r="D28" s="51"/>
-      <c r="E28" s="52"/>
-      <c r="F28" s="52"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="35"/>
-      <c r="I28" s="36"/>
-      <c r="J28" s="33"/>
-      <c r="K28" s="35"/>
-      <c r="L28" s="36"/>
-      <c r="M28" s="33"/>
-      <c r="N28" s="35"/>
-      <c r="O28" s="36"/>
-      <c r="P28" s="33"/>
-      <c r="Q28" s="35"/>
-      <c r="R28" s="36"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="87"/>
+      <c r="E28" s="88"/>
+      <c r="F28" s="88"/>
+      <c r="G28" s="35"/>
+      <c r="H28" s="89"/>
+      <c r="I28" s="90"/>
+      <c r="J28" s="35"/>
+      <c r="K28" s="89"/>
+      <c r="L28" s="90"/>
+      <c r="M28" s="35"/>
+      <c r="N28" s="89"/>
+      <c r="O28" s="90"/>
+      <c r="P28" s="35"/>
+      <c r="Q28" s="89"/>
+      <c r="R28" s="90"/>
     </row>
     <row r="29" spans="2:18" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="49"/>
-      <c r="C29" s="50"/>
+      <c r="B29" s="33"/>
+      <c r="C29" s="34"/>
       <c r="D29" s="85"/>
       <c r="E29" s="86"/>
       <c r="F29" s="86"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="37"/>
-      <c r="I29" s="38"/>
-      <c r="J29" s="34"/>
-      <c r="K29" s="37"/>
-      <c r="L29" s="38"/>
-      <c r="M29" s="34"/>
-      <c r="N29" s="37"/>
-      <c r="O29" s="38"/>
-      <c r="P29" s="34"/>
-      <c r="Q29" s="37"/>
-      <c r="R29" s="38"/>
+      <c r="G29" s="36"/>
+      <c r="H29" s="91"/>
+      <c r="I29" s="92"/>
+      <c r="J29" s="36"/>
+      <c r="K29" s="91"/>
+      <c r="L29" s="92"/>
+      <c r="M29" s="36"/>
+      <c r="N29" s="91"/>
+      <c r="O29" s="92"/>
+      <c r="P29" s="36"/>
+      <c r="Q29" s="91"/>
+      <c r="R29" s="92"/>
     </row>
     <row r="30" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3120,23 +3151,61 @@
     <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="83">
-    <mergeCell ref="J14:K15"/>
-    <mergeCell ref="O14:O15"/>
-    <mergeCell ref="B28:C29"/>
-    <mergeCell ref="B26:C27"/>
-    <mergeCell ref="E4:R7"/>
-    <mergeCell ref="J24:J25"/>
-    <mergeCell ref="K24:L25"/>
-    <mergeCell ref="P24:P25"/>
-    <mergeCell ref="Q24:R25"/>
-    <mergeCell ref="P10:R11"/>
-    <mergeCell ref="P16:Q17"/>
-    <mergeCell ref="Q22:R23"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="G20:I21"/>
-    <mergeCell ref="G12:I13"/>
-    <mergeCell ref="J12:L13"/>
+  <mergeCells count="85">
+    <mergeCell ref="P10:P11"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="M22:M23"/>
+    <mergeCell ref="N22:O23"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="M24:M25"/>
+    <mergeCell ref="N24:O25"/>
+    <mergeCell ref="Q26:R27"/>
+    <mergeCell ref="K28:L29"/>
+    <mergeCell ref="P28:P29"/>
+    <mergeCell ref="Q28:R29"/>
+    <mergeCell ref="M26:M27"/>
+    <mergeCell ref="N26:O27"/>
+    <mergeCell ref="M28:M29"/>
+    <mergeCell ref="N28:O29"/>
+    <mergeCell ref="E16:F17"/>
+    <mergeCell ref="E12:F13"/>
+    <mergeCell ref="E14:F15"/>
+    <mergeCell ref="B22:C23"/>
+    <mergeCell ref="B24:C25"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="B2:D3"/>
+    <mergeCell ref="B20:F21"/>
+    <mergeCell ref="J20:L21"/>
+    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="K22:L23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="H22:I23"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="B18:R19"/>
+    <mergeCell ref="E2:R3"/>
+    <mergeCell ref="E8:F9"/>
+    <mergeCell ref="E10:F11"/>
+    <mergeCell ref="D22:F23"/>
+    <mergeCell ref="G16:H17"/>
+    <mergeCell ref="J16:K17"/>
+    <mergeCell ref="M14:N15"/>
+    <mergeCell ref="P22:P23"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="H26:I27"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="J26:J27"/>
+    <mergeCell ref="J28:J29"/>
+    <mergeCell ref="K26:L27"/>
+    <mergeCell ref="P26:P27"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="H28:I29"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H24:I25"/>
     <mergeCell ref="G14:H15"/>
     <mergeCell ref="P20:R21"/>
     <mergeCell ref="R16:R17"/>
@@ -3153,57 +3222,21 @@
     <mergeCell ref="J8:L9"/>
     <mergeCell ref="M8:O9"/>
     <mergeCell ref="M12:O13"/>
-    <mergeCell ref="M14:N15"/>
-    <mergeCell ref="P22:P23"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="H26:I27"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="J26:J27"/>
-    <mergeCell ref="J28:J29"/>
-    <mergeCell ref="K26:L27"/>
-    <mergeCell ref="P26:P27"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="G28:G29"/>
-    <mergeCell ref="H28:I29"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H24:I25"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="B2:D3"/>
-    <mergeCell ref="B20:F21"/>
-    <mergeCell ref="J20:L21"/>
-    <mergeCell ref="J22:J23"/>
-    <mergeCell ref="K22:L23"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="H22:I23"/>
-    <mergeCell ref="L16:L17"/>
-    <mergeCell ref="B18:R19"/>
-    <mergeCell ref="E2:R3"/>
-    <mergeCell ref="E8:F9"/>
-    <mergeCell ref="E10:F11"/>
-    <mergeCell ref="D22:F23"/>
-    <mergeCell ref="G16:H17"/>
-    <mergeCell ref="J16:K17"/>
-    <mergeCell ref="E16:F17"/>
-    <mergeCell ref="E12:F13"/>
-    <mergeCell ref="E14:F15"/>
-    <mergeCell ref="B22:C23"/>
-    <mergeCell ref="B24:C25"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="Q26:R27"/>
-    <mergeCell ref="K28:L29"/>
-    <mergeCell ref="P28:P29"/>
-    <mergeCell ref="Q28:R29"/>
-    <mergeCell ref="M26:M27"/>
-    <mergeCell ref="N26:O27"/>
-    <mergeCell ref="M28:M29"/>
-    <mergeCell ref="N28:O29"/>
-    <mergeCell ref="M22:M23"/>
-    <mergeCell ref="N22:O23"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="M24:M25"/>
-    <mergeCell ref="N24:O25"/>
+    <mergeCell ref="J14:K15"/>
+    <mergeCell ref="O14:O15"/>
+    <mergeCell ref="B28:C29"/>
+    <mergeCell ref="B26:C27"/>
+    <mergeCell ref="E4:R7"/>
+    <mergeCell ref="J24:J25"/>
+    <mergeCell ref="K24:L25"/>
+    <mergeCell ref="P24:P25"/>
+    <mergeCell ref="Q24:R25"/>
+    <mergeCell ref="P16:Q17"/>
+    <mergeCell ref="Q22:R23"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="G20:I21"/>
+    <mergeCell ref="G12:I13"/>
+    <mergeCell ref="J12:L13"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -3274,7 +3307,7 @@
         <v>32</v>
       </c>
       <c r="D5" s="9"/>
-      <c r="F5" s="132">
+      <c r="F5" s="123">
         <f>SUM(F7:F22)</f>
         <v>7.05</v>
       </c>
@@ -3286,7 +3319,7 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="F6" s="133"/>
+      <c r="F6" s="124"/>
       <c r="H6" s="13" t="s">
         <v>50</v>
       </c>
@@ -3414,7 +3447,7 @@
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
       <c r="F14" s="17"/>
-      <c r="H14" s="134">
+      <c r="H14" s="125">
         <f>J12+I9</f>
         <v>0.1187</v>
       </c>
@@ -3434,7 +3467,7 @@
       <c r="F15" s="16">
         <v>0.7</v>
       </c>
-      <c r="H15" s="134"/>
+      <c r="H15" s="125"/>
     </row>
     <row r="16" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A16" s="19"/>

</xml_diff>